<commit_message>
un poco de todo
</commit_message>
<xml_diff>
--- a/2026/2DE MAYO/Septiembre/2DEDMAYO-Septiembre.xlsx
+++ b/2026/2DE MAYO/Septiembre/2DEDMAYO-Septiembre.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\2026\2DE MAYO\Septiembre\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistemax\Desktop\rc-consorcio2025\2026\2DE MAYO\Septiembre\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FDD9C0E-F023-47F0-A26C-B392A0C84D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126C1EF7-3BAB-4051-A92D-138680B95BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="850" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -19,14 +19,19 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">PRORRATEO!$A$1:$O$36</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$E$104</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$E$101</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="142">
   <si>
     <t>LIQUIDACION DE EXPENSAS</t>
   </si>
@@ -394,45 +399,15 @@
     <t>Intereses generados</t>
   </si>
   <si>
-    <t>Transf 04/08</t>
-  </si>
-  <si>
-    <t>Transf 05/08</t>
-  </si>
-  <si>
-    <t>Transf 12/08</t>
-  </si>
-  <si>
-    <t>Debito 10/08</t>
-  </si>
-  <si>
-    <t>Debito 12/08</t>
-  </si>
-  <si>
     <t>Reemplazo Sra. Silvana - Vacaciones Sra. Lucia</t>
   </si>
   <si>
-    <t>Seguro Sra. Silvana</t>
-  </si>
-  <si>
-    <t>Arreglo de camaras</t>
-  </si>
-  <si>
     <t xml:space="preserve">Saldo inicial FCI </t>
   </si>
   <si>
-    <t>Transf 24/08</t>
-  </si>
-  <si>
-    <t>Transf 31/08</t>
-  </si>
-  <si>
     <t>Della Maggora</t>
   </si>
   <si>
-    <t xml:space="preserve">Caja chicha entregada a Lucia </t>
-  </si>
-  <si>
     <t>VTO 16/10</t>
   </si>
   <si>
@@ -464,6 +439,24 @@
   </si>
   <si>
     <t>Transf 09/09</t>
+  </si>
+  <si>
+    <t>Transf 04/09</t>
+  </si>
+  <si>
+    <t>Debito 14/09</t>
+  </si>
+  <si>
+    <t>Debito 08/09</t>
+  </si>
+  <si>
+    <t>Debito 10/09</t>
+  </si>
+  <si>
+    <t>Transf 10/09</t>
+  </si>
+  <si>
+    <t>Transf 30/09</t>
   </si>
 </sst>
 </file>
@@ -481,7 +474,7 @@
     <numFmt numFmtId="168" formatCode="_-[$$-2C0A]\ * #,##0.00_-;\-[$$-2C0A]\ * #,##0.00_-;_-[$$-2C0A]\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="169" formatCode="0.000"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +650,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -1249,7 +1249,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="218">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1290,9 +1290,6 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="44" fontId="9" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1501,8 +1498,51 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="18" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="16" fontId="18" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1516,131 +1556,26 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="18" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" fontId="18" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1650,8 +1585,77 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="44" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="23" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -1730,9 +1734,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1770,9 +1774,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1805,9 +1809,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1840,9 +1861,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2016,75 +2054,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M108"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M105"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.5546875" customWidth="1"/>
-    <col min="2" max="2" width="24.6640625" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.7109375" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="18.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="14"/>
-      <c r="B1" s="176" t="s">
-        <v>136</v>
-      </c>
-      <c r="C1" s="176"/>
-      <c r="D1" s="176"/>
-      <c r="E1" s="51"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="169" t="s">
+        <v>126</v>
+      </c>
+      <c r="C1" s="169"/>
+      <c r="D1" s="169"/>
+      <c r="E1" s="50"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
-      <c r="E2" s="53"/>
-    </row>
-    <row r="3" spans="1:5" ht="70.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="52"/>
+    </row>
+    <row r="3" spans="1:5" ht="70.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="15"/>
-      <c r="B3" s="177" t="s">
+      <c r="B3" s="172" t="s">
         <v>95</v>
       </c>
-      <c r="C3" s="177"/>
-      <c r="D3" s="177"/>
-      <c r="E3" s="178"/>
-    </row>
-    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="172"/>
+      <c r="D3" s="172"/>
+      <c r="E3" s="173"/>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="54" t="s">
+      <c r="B4" s="53" t="s">
         <v>31</v>
       </c>
       <c r="C4" s="19"/>
       <c r="D4" s="19"/>
       <c r="E4" s="20"/>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
         <v>111</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="C5" s="16"/>
-      <c r="D5" s="52" t="s">
+      <c r="D5" s="51" t="s">
         <v>23</v>
       </c>
       <c r="E5" s="17"/>
     </row>
-    <row r="6" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B6" s="19"/>
       <c r="C6" s="19"/>
@@ -2093,57 +2131,57 @@
       </c>
       <c r="E6" s="20"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="180" t="s">
-        <v>135</v>
-      </c>
-      <c r="C8" s="180"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="180"/>
-      <c r="C9" s="180"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B10" s="180"/>
-      <c r="C10" s="180"/>
-    </row>
-    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="179" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="175" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="175"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="175"/>
+      <c r="C9" s="175"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="175"/>
+      <c r="C10" s="175"/>
+    </row>
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="174" t="s">
         <v>87</v>
       </c>
-      <c r="B13" s="179"/>
-      <c r="C13" s="179"/>
-      <c r="D13" s="179"/>
-      <c r="E13" s="179"/>
-    </row>
-    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="179"/>
-      <c r="B14" s="179"/>
-      <c r="C14" s="179"/>
-      <c r="D14" s="179"/>
-      <c r="E14" s="179"/>
-    </row>
-    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="179"/>
-      <c r="B15" s="179"/>
-      <c r="C15" s="179"/>
-      <c r="D15" s="179"/>
-      <c r="E15" s="179"/>
-    </row>
-    <row r="16" spans="1:5" ht="127.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="179"/>
-      <c r="B16" s="179"/>
-      <c r="C16" s="179"/>
-      <c r="D16" s="179"/>
-      <c r="E16" s="179"/>
-    </row>
-    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="174"/>
+      <c r="C13" s="174"/>
+      <c r="D13" s="174"/>
+      <c r="E13" s="174"/>
+    </row>
+    <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="174"/>
+      <c r="B14" s="174"/>
+      <c r="C14" s="174"/>
+      <c r="D14" s="174"/>
+      <c r="E14" s="174"/>
+    </row>
+    <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="174"/>
+      <c r="B15" s="174"/>
+      <c r="C15" s="174"/>
+      <c r="D15" s="174"/>
+      <c r="E15" s="174"/>
+    </row>
+    <row r="16" spans="1:5" ht="127.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="174"/>
+      <c r="B16" s="174"/>
+      <c r="C16" s="174"/>
+      <c r="D16" s="174"/>
+      <c r="E16" s="174"/>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
     </row>
-    <row r="19" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>9</v>
       </c>
@@ -2152,7 +2190,7 @@
       <c r="D20" s="8"/>
       <c r="E20" s="13"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="27" t="s">
         <v>27</v>
       </c>
@@ -2161,217 +2199,215 @@
       <c r="D21" s="26"/>
       <c r="E21" s="26"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="C22" s="5"/>
-      <c r="D22" s="134">
-        <v>1506395.81</v>
+      <c r="D22" s="133">
+        <v>1429122.26</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>89</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
-      <c r="D23" s="134">
-        <v>-372832.81</v>
+      <c r="D23" s="133">
+        <v>-353707.26</v>
       </c>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>90</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
-      <c r="D24" s="134">
+      <c r="D24" s="133">
         <v>0</v>
       </c>
       <c r="E24" s="5"/>
     </row>
-    <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="44" t="s">
+    <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="44"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="135">
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="134">
         <f>SUM(D22:D24)</f>
-        <v>1133563</v>
-      </c>
-      <c r="E25" s="85"/>
+        <v>1075415</v>
+      </c>
+      <c r="E25" s="84"/>
       <c r="G25" s="21"/>
     </row>
-    <row r="26" spans="1:7" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>34</v>
       </c>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
-      <c r="D26" s="134"/>
+      <c r="D26" s="133"/>
       <c r="E26" s="5"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="23" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
-      <c r="D27" s="134">
-        <v>211200</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="44" t="s">
+      <c r="D27" s="133">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5"/>
+    </row>
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="136">
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="135">
         <f>SUM(D26:D27)</f>
-        <v>211200</v>
-      </c>
-      <c r="E28" s="85"/>
-    </row>
-    <row r="29" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="E28" s="84"/>
+    </row>
+    <row r="29" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="24" t="s">
         <v>1</v>
       </c>
       <c r="B29" s="24"/>
       <c r="C29" s="24"/>
-      <c r="D29" s="137"/>
-      <c r="E29" s="86">
+      <c r="D29" s="136"/>
+      <c r="E29" s="85">
         <f>D25+D28</f>
-        <v>1344763</v>
+        <v>1075415</v>
       </c>
       <c r="F29" s="21"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="27" t="s">
         <v>18</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
-      <c r="D30" s="138"/>
-      <c r="E30" s="87"/>
-    </row>
-    <row r="31" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D30" s="137"/>
+      <c r="E30" s="86"/>
+    </row>
+    <row r="31" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="170" t="s">
         <v>117</v>
       </c>
       <c r="B31" s="171"/>
-      <c r="C31" s="41"/>
-      <c r="D31" s="134">
+      <c r="C31" s="40"/>
+      <c r="D31" s="133">
         <v>50000</v>
       </c>
-      <c r="E31" s="131" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E31" s="130" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="24" t="s">
         <v>15</v>
       </c>
       <c r="B32" s="24"/>
       <c r="C32" s="24"/>
-      <c r="D32" s="146"/>
-      <c r="E32" s="88">
+      <c r="D32" s="145"/>
+      <c r="E32" s="87">
         <f>SUM(D31:D31)</f>
         <v>50000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="27" t="s">
         <v>25</v>
       </c>
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
-      <c r="D33" s="147"/>
-      <c r="E33" s="89"/>
-    </row>
-    <row r="34" spans="1:7" s="30" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="181" t="s">
+      <c r="D33" s="146"/>
+      <c r="E33" s="88"/>
+    </row>
+    <row r="34" spans="1:7" s="30" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="176" t="s">
         <v>119</v>
       </c>
-      <c r="B34" s="182"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="172">
+      <c r="B34" s="177"/>
+      <c r="C34" s="41"/>
+      <c r="D34" s="165">
         <v>76880</v>
       </c>
-      <c r="E34" s="174" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="183"/>
-      <c r="B35" s="184"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="173"/>
-      <c r="E35" s="175"/>
-    </row>
-    <row r="36" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E34" s="167" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="42" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="178"/>
+      <c r="B35" s="179"/>
+      <c r="C35" s="41"/>
+      <c r="D35" s="166"/>
+      <c r="E35" s="168"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="24" t="s">
         <v>2</v>
       </c>
       <c r="B36" s="24"/>
       <c r="C36" s="24"/>
-      <c r="D36" s="146"/>
-      <c r="E36" s="58">
+      <c r="D36" s="145"/>
+      <c r="E36" s="57">
         <f>SUM(D34:D35)</f>
         <v>76880</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="90"/>
-      <c r="C37" s="90"/>
-      <c r="D37" s="148"/>
-      <c r="E37" s="140"/>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B37" s="89"/>
+      <c r="C37" s="89"/>
+      <c r="D37" s="147"/>
+      <c r="E37" s="139"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="5"/>
-      <c r="C38" s="41"/>
-      <c r="D38" s="216">
+      <c r="C38" s="40"/>
+      <c r="D38" s="138">
         <v>868381.3</v>
       </c>
-      <c r="E38" s="131" t="s">
-        <v>143</v>
-      </c>
-      <c r="G38" s="75"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E38" s="130" t="s">
+        <v>133</v>
+      </c>
+      <c r="G38" s="74"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>98</v>
       </c>
       <c r="C39" s="5"/>
-      <c r="D39" s="216">
+      <c r="D39" s="138">
         <v>67787.78</v>
       </c>
-      <c r="E39" s="94" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E39" s="93" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="str">
         <f>A39</f>
         <v>Sindicatos mes de SEPTIEMBRE</v>
@@ -2380,15 +2416,15 @@
         <v>97</v>
       </c>
       <c r="C40" s="5"/>
-      <c r="D40" s="216">
+      <c r="D40" s="138">
         <v>123080.68</v>
       </c>
-      <c r="E40" s="95" t="str">
+      <c r="E40" s="94" t="str">
         <f>E39</f>
-        <v>Debito 12/08</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+        <v>Debito 14/09</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="str">
         <f>A40</f>
         <v>Sindicatos mes de SEPTIEMBRE</v>
@@ -2397,608 +2433,586 @@
         <v>96</v>
       </c>
       <c r="C41" s="5"/>
-      <c r="D41" s="216">
+      <c r="D41" s="138">
         <v>7531.98</v>
       </c>
-      <c r="E41" s="96" t="str">
+      <c r="E41" s="95" t="str">
         <f>E40</f>
-        <v>Debito 12/08</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>Debito 14/09</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B42" s="90"/>
-      <c r="C42" s="90"/>
-      <c r="D42" s="149"/>
-      <c r="E42" s="58">
+      <c r="B42" s="89"/>
+      <c r="C42" s="89"/>
+      <c r="D42" s="148"/>
+      <c r="E42" s="57">
         <f>SUM(D38:D41)</f>
         <v>1066781.74</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B43" s="90"/>
-      <c r="C43" s="90"/>
-      <c r="D43" s="148"/>
-      <c r="E43" s="140"/>
-    </row>
-    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="89"/>
+      <c r="C43" s="89"/>
+      <c r="D43" s="147"/>
+      <c r="E43" s="139"/>
+    </row>
+    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>91</v>
       </c>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
-      <c r="D44" s="139">
-        <v>439936.38</v>
-      </c>
-      <c r="E44" s="94" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="123" t="s">
+      <c r="D44" s="138">
+        <v>417256.82</v>
+      </c>
+      <c r="E44" s="93" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="122" t="s">
         <v>92</v>
       </c>
-      <c r="B45" s="124"/>
+      <c r="B45" s="123"/>
       <c r="C45" s="5"/>
-      <c r="D45" s="216">
+      <c r="D45" s="138">
         <v>391412.67</v>
       </c>
-      <c r="E45" s="94" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E45" s="93" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B46" s="24"/>
       <c r="C46" s="24"/>
-      <c r="D46" s="150"/>
-      <c r="E46" s="58">
+      <c r="D46" s="149"/>
+      <c r="E46" s="57">
         <f>SUM(D44:D45)</f>
-        <v>831349.05</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>808669.49</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="27"/>
       <c r="B47" s="24"/>
       <c r="C47" s="24"/>
-      <c r="D47" s="146"/>
-      <c r="E47" s="141"/>
-    </row>
-    <row r="48" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="97" t="s">
+      <c r="D47" s="145"/>
+      <c r="E47" s="140"/>
+    </row>
+    <row r="48" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="96" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="93"/>
+      <c r="B48" s="92"/>
       <c r="C48" s="5"/>
-      <c r="D48" s="139">
-        <v>20417</v>
-      </c>
-      <c r="E48" s="94" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="97" t="s">
-        <v>144</v>
-      </c>
-      <c r="B49" s="93"/>
+      <c r="D48" s="138">
+        <v>20849.400000000001</v>
+      </c>
+      <c r="E48" s="93" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="96" t="s">
+        <v>134</v>
+      </c>
+      <c r="B49" s="92"/>
       <c r="C49" s="5"/>
-      <c r="D49" s="216">
+      <c r="D49" s="138">
         <v>180000</v>
       </c>
-      <c r="E49" s="217" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="97" t="s">
+      <c r="E49" s="164" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="96" t="s">
         <v>113</v>
       </c>
-      <c r="B50" s="93"/>
+      <c r="B50" s="92"/>
       <c r="C50" s="5"/>
-      <c r="D50" s="216">
+      <c r="D50" s="138">
         <v>126000</v>
       </c>
-      <c r="E50" s="131" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="166" t="s">
+      <c r="E50" s="130" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="180" t="s">
         <v>118</v>
       </c>
-      <c r="B51" s="167"/>
+      <c r="B51" s="181"/>
       <c r="C51" s="5"/>
-      <c r="D51" s="216">
+      <c r="D51" s="138">
         <v>833334</v>
       </c>
-      <c r="E51" s="131" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E51" s="130" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="24" t="s">
         <v>8</v>
       </c>
       <c r="B52" s="27"/>
       <c r="C52" s="27"/>
       <c r="D52" s="26"/>
-      <c r="E52" s="142">
+      <c r="E52" s="141">
         <f>SUM(D48:D51)</f>
-        <v>1159751</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>1160183.3999999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B53" s="49"/>
+      <c r="B53" s="48"/>
       <c r="C53" s="24"/>
-      <c r="D53" s="137"/>
-      <c r="E53" s="91"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="D53" s="136"/>
+      <c r="E53" s="90"/>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>45</v>
       </c>
       <c r="B54" s="5"/>
       <c r="C54" s="5"/>
-      <c r="D54" s="139">
+      <c r="D54" s="138">
         <v>69000</v>
       </c>
-      <c r="E54" s="92"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="E54" s="91"/>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B55" s="5"/>
       <c r="C55" s="5"/>
-      <c r="D55" s="139">
-        <f>635+75121.34</f>
-        <v>75756.34</v>
+      <c r="D55" s="138">
+        <v>72086.2</v>
       </c>
       <c r="E55" s="31"/>
     </row>
-    <row r="56" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="40" t="s">
+    <row r="56" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="B56" s="40"/>
-      <c r="C56" s="40"/>
-      <c r="D56" s="63"/>
-      <c r="E56" s="58">
+      <c r="B56" s="39"/>
+      <c r="C56" s="39"/>
+      <c r="D56" s="62"/>
+      <c r="E56" s="57">
         <f>SUM(D54:D55)</f>
-        <v>144756.34</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+        <v>141086.20000000001</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5"/>
       <c r="B57" s="5"/>
       <c r="C57" s="5"/>
-      <c r="D57" s="57"/>
-      <c r="E57" s="64"/>
-    </row>
-    <row r="58" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D57" s="56"/>
+      <c r="E57" s="63"/>
+    </row>
+    <row r="58" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="25" t="s">
         <v>116</v>
       </c>
       <c r="B58" s="25"/>
       <c r="C58" s="25"/>
-      <c r="D58" s="65"/>
-      <c r="E58" s="66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D58" s="64"/>
+      <c r="E58" s="65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="1"/>
-      <c r="D59" s="67"/>
-      <c r="E59" s="68"/>
+      <c r="D59" s="66"/>
+      <c r="E59" s="67"/>
       <c r="F59" s="33"/>
     </row>
-    <row r="60" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B60" s="9"/>
       <c r="C60" s="4"/>
-      <c r="D60" s="69"/>
-      <c r="E60" s="70">
+      <c r="D60" s="68"/>
+      <c r="E60" s="69">
         <f>(SUM(E28:E58))</f>
-        <v>4674281.13</v>
-      </c>
-      <c r="F60" s="84"/>
+        <v>4379015.830000001</v>
+      </c>
+      <c r="F60" s="83"/>
       <c r="G60" s="33"/>
-      <c r="H60" s="75"/>
-      <c r="I60" s="75"/>
-      <c r="J60" s="75"/>
-      <c r="K60" s="75"/>
-      <c r="L60" s="75"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="D61" s="67"/>
-      <c r="E61" s="67"/>
-      <c r="H61" s="75"/>
-      <c r="I61" s="75"/>
-      <c r="J61" s="75"/>
-      <c r="K61" s="75"/>
-      <c r="L61" s="75"/>
-    </row>
-    <row r="62" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D62" s="67"/>
-      <c r="E62" s="67"/>
-      <c r="H62" s="98"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="H60" s="74"/>
+      <c r="I60" s="74"/>
+      <c r="J60" s="74"/>
+      <c r="K60" s="74"/>
+      <c r="L60" s="74"/>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="D61" s="66"/>
+      <c r="E61" s="66"/>
+      <c r="H61" s="74"/>
+      <c r="I61" s="74"/>
+      <c r="J61" s="74"/>
+      <c r="K61" s="74"/>
+      <c r="L61" s="74"/>
+    </row>
+    <row r="62" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D62" s="66"/>
+      <c r="E62" s="66"/>
+      <c r="H62" s="97"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="10" t="s">
         <v>35</v>
       </c>
       <c r="B63" s="11"/>
       <c r="C63" s="12"/>
-      <c r="D63" s="71"/>
-      <c r="E63" s="72"/>
-    </row>
-    <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="166"/>
-      <c r="B64" s="167"/>
+      <c r="D63" s="70"/>
+      <c r="E63" s="71"/>
+    </row>
+    <row r="64" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="180"/>
+      <c r="B64" s="181"/>
       <c r="C64" s="5"/>
-      <c r="D64" s="61"/>
-      <c r="E64" s="59"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A65" s="166"/>
-      <c r="B65" s="167"/>
+      <c r="D64" s="60"/>
+      <c r="E64" s="58"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="180"/>
+      <c r="B65" s="181"/>
       <c r="C65" s="5"/>
-      <c r="D65" s="61"/>
-      <c r="E65" s="59"/>
-    </row>
-    <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D65" s="60"/>
+      <c r="E65" s="58"/>
+    </row>
+    <row r="66" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="170"/>
       <c r="B66" s="171"/>
       <c r="C66" s="5"/>
-      <c r="D66" s="61"/>
-      <c r="E66" s="59"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A67" s="60"/>
-      <c r="B67" s="62"/>
+      <c r="D66" s="60"/>
+      <c r="E66" s="58"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="59"/>
+      <c r="B67" s="61"/>
       <c r="C67" s="5"/>
-      <c r="D67" s="61"/>
-      <c r="E67" s="59"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A68" s="38"/>
-      <c r="B68" s="37"/>
-      <c r="C68" s="37"/>
-      <c r="D68" s="155"/>
-      <c r="E68" s="45">
+      <c r="D67" s="60"/>
+      <c r="E67" s="58"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="37"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="36"/>
+      <c r="D68" s="154"/>
+      <c r="E68" s="44">
         <f>SUM(D64:D67)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D69" s="67"/>
-    </row>
-    <row r="70" spans="1:5" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D70" s="67"/>
-    </row>
-    <row r="71" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="132" t="s">
+    <row r="69" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D69" s="66"/>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D70" s="66"/>
+    </row>
+    <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="131" t="s">
         <v>115</v>
       </c>
-      <c r="B71" s="133"/>
-      <c r="C71" s="133"/>
-      <c r="D71" s="156"/>
-      <c r="E71" s="143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D72" s="67"/>
-    </row>
-    <row r="73" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B71" s="132"/>
+      <c r="C71" s="132"/>
+      <c r="D71" s="155"/>
+      <c r="E71" s="142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D72" s="66"/>
+    </row>
+    <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B73" s="9"/>
       <c r="C73" s="4"/>
-      <c r="D73" s="69"/>
-      <c r="E73" s="50">
+      <c r="D73" s="68"/>
+      <c r="E73" s="49">
         <f>E68+E71</f>
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D74" s="67"/>
-    </row>
-    <row r="75" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="55" t="s">
+    <row r="74" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D74" s="66"/>
+    </row>
+    <row r="75" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="56">
+      <c r="B75" s="55">
         <f>E60</f>
-        <v>4674281.13</v>
-      </c>
-      <c r="D75" s="67"/>
-    </row>
-    <row r="76" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="55" t="s">
+        <v>4379015.830000001</v>
+      </c>
+      <c r="D75" s="66"/>
+    </row>
+    <row r="76" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="B76" s="56">
+      <c r="B76" s="55">
         <f>E60-E58</f>
-        <v>4674281.13</v>
-      </c>
-      <c r="D76" s="67"/>
-    </row>
-    <row r="77" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="55" t="s">
+        <v>4379015.830000001</v>
+      </c>
+      <c r="D76" s="66"/>
+    </row>
+    <row r="77" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="B77" s="56">
+      <c r="B77" s="55">
         <f>E73-E71</f>
         <v>0</v>
       </c>
-      <c r="D77" s="67"/>
-    </row>
-    <row r="78" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="55" t="s">
+      <c r="D77" s="66"/>
+    </row>
+    <row r="78" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="B78" s="56">
+      <c r="B78" s="55">
         <f>E73</f>
         <v>0</v>
       </c>
-      <c r="D78" s="67"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="D79" s="67"/>
-    </row>
-    <row r="80" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D80" s="67"/>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="151" t="s">
+      <c r="D78" s="66"/>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D79" s="66"/>
+    </row>
+    <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D80" s="66"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="150" t="s">
         <v>105</v>
       </c>
-      <c r="B81" s="152">
-        <v>162946.62000000011</v>
-      </c>
-      <c r="D81" s="67"/>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="125" t="s">
+      <c r="B81" s="151">
+        <v>100489.93000000011</v>
+      </c>
+      <c r="D81" s="66"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="124" t="s">
         <v>108</v>
       </c>
-      <c r="B82" s="126">
+      <c r="B82" s="125">
         <f>PRORRATEO!G38</f>
-        <v>226480.31</v>
+        <v>302032.34000000003</v>
       </c>
       <c r="C82" s="22"/>
-      <c r="D82" s="67"/>
-      <c r="E82" s="76"/>
-      <c r="F82" s="77"/>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="153" t="s">
-        <v>128</v>
-      </c>
-      <c r="B83" s="144">
-        <v>-5837</v>
+      <c r="D82" s="66"/>
+      <c r="E82" s="75"/>
+      <c r="F82" s="76"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="152" t="s">
+        <v>130</v>
+      </c>
+      <c r="B83" s="143">
+        <v>-133100</v>
       </c>
       <c r="C83" s="22"/>
-      <c r="D83" s="67"/>
-      <c r="E83" s="76"/>
-      <c r="F83" s="77"/>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="153" t="s">
-        <v>129</v>
-      </c>
-      <c r="B84" s="144">
-        <v>-150000</v>
+      <c r="D83" s="66"/>
+      <c r="E83" s="75"/>
+      <c r="F83" s="76"/>
+    </row>
+    <row r="84" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="126" t="s">
+        <v>37</v>
+      </c>
+      <c r="B84" s="127">
+        <f>SUM(B81:C83)</f>
+        <v>269422.27000000014</v>
       </c>
       <c r="C84" s="22"/>
-      <c r="D84" s="67"/>
-      <c r="E84" s="76"/>
-      <c r="F84" s="77"/>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="153" t="s">
-        <v>140</v>
-      </c>
-      <c r="B85" s="144">
-        <v>-133100</v>
-      </c>
-      <c r="C85" s="22"/>
-      <c r="D85" s="67"/>
-      <c r="E85" s="76"/>
-      <c r="F85" s="77"/>
-    </row>
-    <row r="86" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A86" s="127" t="s">
+      <c r="D84" s="66"/>
+    </row>
+    <row r="85" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A85"/>
+      <c r="B85" s="32"/>
+      <c r="C85" s="29"/>
+      <c r="D85" s="66"/>
+    </row>
+    <row r="86" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A86" s="77" t="s">
+        <v>43</v>
+      </c>
+      <c r="B86" s="163">
+        <v>427006.25000000326</v>
+      </c>
+      <c r="C86" s="29"/>
+      <c r="D86" s="216"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="41" t="s">
+        <v>39</v>
+      </c>
+      <c r="B87" s="156">
+        <f>-B76</f>
+        <v>-4379015.830000001</v>
+      </c>
+      <c r="D87" s="66"/>
+      <c r="E87" s="33"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B88" s="81">
+        <f>-B77</f>
+        <v>0</v>
+      </c>
+      <c r="D88" s="66"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" s="41" t="s">
+        <v>42</v>
+      </c>
+      <c r="B89" s="81">
+        <f>B100</f>
+        <v>0</v>
+      </c>
+      <c r="D89" s="66"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" s="41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B90" s="82">
+        <f>PRORRATEO!G37</f>
+        <v>4119366.350000001</v>
+      </c>
+      <c r="D90" s="66"/>
+    </row>
+    <row r="91" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="B86" s="128">
-        <f>SUM(B81:C85)</f>
-        <v>100489.93000000011</v>
-      </c>
-      <c r="C86" s="22"/>
-    </row>
-    <row r="87" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A87"/>
-      <c r="B87" s="32"/>
-      <c r="C87" s="29"/>
-      <c r="D87"/>
-    </row>
-    <row r="88" spans="1:6" s="30" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="78" t="s">
-        <v>43</v>
-      </c>
-      <c r="B88" s="164">
-        <v>479322.8200000017</v>
-      </c>
-      <c r="C88" s="29"/>
-      <c r="D88" s="36"/>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="42" t="s">
-        <v>39</v>
-      </c>
-      <c r="B89" s="157">
-        <f>-B76</f>
-        <v>-4674281.13</v>
-      </c>
-      <c r="E89" s="33"/>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="42" t="s">
-        <v>40</v>
-      </c>
-      <c r="B90" s="82">
-        <f>-B77</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="42" t="s">
-        <v>134</v>
-      </c>
-      <c r="B91" s="165">
-        <v>80000</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B92" s="82">
-        <f>B103</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="42" t="s">
-        <v>41</v>
-      </c>
-      <c r="B93" s="83">
-        <f>PRORRATEO!G37</f>
-        <v>4254804.3600000013</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A94" s="80" t="s">
-        <v>37</v>
-      </c>
-      <c r="B94" s="81">
-        <f>SUM(B88:C93)</f>
-        <v>139846.05000000261</v>
-      </c>
-      <c r="D94" s="32"/>
-      <c r="E94" s="33"/>
-    </row>
-    <row r="95" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A95" s="79"/>
-      <c r="B95" s="79"/>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="162" t="s">
-        <v>130</v>
-      </c>
-      <c r="B96" s="158">
-        <v>872509.82</v>
-      </c>
-    </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A97" s="160" t="s">
+      <c r="B91" s="80">
+        <f>SUM(B86:C90)</f>
+        <v>167356.77000000328</v>
+      </c>
+      <c r="D91" s="217"/>
+      <c r="E91" s="33"/>
+    </row>
+    <row r="92" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="78"/>
+      <c r="B92" s="78"/>
+      <c r="D92" s="66"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" s="161" t="s">
+        <v>123</v>
+      </c>
+      <c r="B93" s="157">
+        <v>885117.96</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" s="159" t="s">
         <v>121</v>
       </c>
-      <c r="B97" s="161">
-        <f>885117.96-872509.82</f>
-        <v>12608.140000000014</v>
-      </c>
-    </row>
-    <row r="98" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="163" t="s">
+      <c r="B94" s="160">
+        <f>B95-B93</f>
+        <v>14104.560000000056</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="162" t="s">
         <v>120</v>
       </c>
-      <c r="B98" s="159">
-        <f>885117.96</f>
-        <v>885117.96</v>
-      </c>
-      <c r="D98" s="33"/>
-    </row>
-    <row r="99" spans="1:13" ht="34.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A100" s="169" t="s">
+      <c r="B95" s="158">
+        <v>899222.52</v>
+      </c>
+      <c r="D95" s="33"/>
+    </row>
+    <row r="96" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A97" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="B100" s="169"/>
-      <c r="C100" s="169"/>
-    </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A101" s="169"/>
-      <c r="B101" s="169"/>
-      <c r="C101" s="169"/>
-    </row>
-    <row r="102" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="73"/>
-      <c r="B102" s="28"/>
-      <c r="C102" s="28">
+      <c r="B97" s="183"/>
+      <c r="C97" s="183"/>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A98" s="183"/>
+      <c r="B98" s="183"/>
+      <c r="C98" s="183"/>
+    </row>
+    <row r="99" spans="1:13" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="72"/>
+      <c r="B99" s="28"/>
+      <c r="C99" s="28">
         <v>40000</v>
       </c>
-      <c r="E102" s="84"/>
-    </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A103" s="34" t="s">
+      <c r="E99" s="83"/>
+    </row>
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A100" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="B103" s="74">
-        <f>SUM(B102:B102)</f>
-        <v>0</v>
-      </c>
-      <c r="C103" s="35"/>
-    </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="M104" s="7"/>
-    </row>
-    <row r="105" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A105" s="168"/>
-      <c r="B105" s="168"/>
-      <c r="C105" s="168"/>
-      <c r="D105" s="168"/>
-      <c r="E105" s="168"/>
-    </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A106" s="168"/>
-      <c r="B106" s="168"/>
-      <c r="C106" s="168"/>
-      <c r="D106" s="168"/>
-      <c r="E106" s="168"/>
-    </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A107" s="168"/>
-      <c r="B107" s="168"/>
-      <c r="C107" s="168"/>
-      <c r="D107" s="168"/>
-      <c r="E107" s="168"/>
-    </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A108" s="168"/>
-      <c r="B108" s="168"/>
-      <c r="C108" s="168"/>
-      <c r="D108" s="168"/>
-      <c r="E108" s="168"/>
+      <c r="B100" s="73">
+        <f>SUM(B99:B99)</f>
+        <v>0</v>
+      </c>
+      <c r="C100" s="35"/>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="M101" s="7"/>
+    </row>
+    <row r="102" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="182"/>
+      <c r="B102" s="182"/>
+      <c r="C102" s="182"/>
+      <c r="D102" s="182"/>
+      <c r="E102" s="182"/>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A103" s="182"/>
+      <c r="B103" s="182"/>
+      <c r="C103" s="182"/>
+      <c r="D103" s="182"/>
+      <c r="E103" s="182"/>
+    </row>
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A104" s="182"/>
+      <c r="B104" s="182"/>
+      <c r="C104" s="182"/>
+      <c r="D104" s="182"/>
+      <c r="E104" s="182"/>
+    </row>
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A105" s="182"/>
+      <c r="B105" s="182"/>
+      <c r="C105" s="182"/>
+      <c r="D105" s="182"/>
+      <c r="E105" s="182"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A51:B51"/>
+    <mergeCell ref="A102:E105"/>
+    <mergeCell ref="A97:C98"/>
+    <mergeCell ref="A65:B65"/>
+    <mergeCell ref="A64:B64"/>
+    <mergeCell ref="A66:B66"/>
     <mergeCell ref="D34:D35"/>
     <mergeCell ref="E34:E35"/>
     <mergeCell ref="B1:D1"/>
@@ -3007,12 +3021,6 @@
     <mergeCell ref="A13:E16"/>
     <mergeCell ref="B8:C10"/>
     <mergeCell ref="A34:B35"/>
-    <mergeCell ref="A51:B51"/>
-    <mergeCell ref="A105:E108"/>
-    <mergeCell ref="A100:C101"/>
-    <mergeCell ref="A65:B65"/>
-    <mergeCell ref="A64:B64"/>
-    <mergeCell ref="A66:B66"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -3023,74 +3031,74 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="6.5546875" customWidth="1"/>
-    <col min="3" max="3" width="20.44140625" customWidth="1"/>
-    <col min="4" max="4" width="22.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" customWidth="1"/>
+    <col min="1" max="1" width="4.28515625" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="22.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
     <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" customWidth="1"/>
-    <col min="10" max="11" width="9.5546875" customWidth="1"/>
-    <col min="12" max="13" width="12.44140625" customWidth="1"/>
-    <col min="14" max="14" width="14.6640625" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" customWidth="1"/>
-    <col min="16" max="16" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.5703125" customWidth="1"/>
+    <col min="10" max="11" width="9.5703125" customWidth="1"/>
+    <col min="12" max="13" width="12.42578125" customWidth="1"/>
+    <col min="14" max="14" width="14.7109375" customWidth="1"/>
+    <col min="15" max="15" width="14.28515625" customWidth="1"/>
+    <col min="16" max="16" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="12.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
-      <c r="E1" s="185"/>
-      <c r="F1" s="185"/>
-      <c r="G1" s="185"/>
-      <c r="H1" s="185"/>
-      <c r="I1" s="185"/>
-      <c r="J1" s="185"/>
-      <c r="K1" s="185"/>
-      <c r="L1" s="185"/>
-      <c r="M1" s="185"/>
-      <c r="N1" s="185"/>
+      <c r="E1" s="197"/>
+      <c r="F1" s="197"/>
+      <c r="G1" s="197"/>
+      <c r="H1" s="197"/>
+      <c r="I1" s="197"/>
+      <c r="J1" s="197"/>
+      <c r="K1" s="197"/>
+      <c r="L1" s="197"/>
+      <c r="M1" s="197"/>
+      <c r="N1" s="197"/>
       <c r="O1" s="6"/>
     </row>
-    <row r="2" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="211">
-        <v>0</v>
-      </c>
-      <c r="E2" s="211"/>
+      <c r="D2" s="188">
+        <v>0</v>
+      </c>
+      <c r="E2" s="188"/>
       <c r="F2" s="6"/>
-      <c r="G2" s="211"/>
-      <c r="H2" s="211"/>
-      <c r="I2" s="211"/>
+      <c r="G2" s="188"/>
+      <c r="H2" s="188"/>
+      <c r="I2" s="188"/>
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
       <c r="L2" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="M2" s="210">
+      <c r="M2" s="187">
         <f>Q2</f>
-        <v>4387120.93</v>
-      </c>
-      <c r="N2" s="210"/>
-      <c r="O2" s="43"/>
+        <v>4379015.830000001</v>
+      </c>
+      <c r="N2" s="187"/>
+      <c r="O2" s="42"/>
       <c r="P2" s="21"/>
       <c r="Q2">
-        <v>4387120.93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="12.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>4379015.830000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="12.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -3104,265 +3112,265 @@
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="6"/>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-    </row>
-    <row r="4" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="194" t="str">
+      <c r="N3" s="45"/>
+      <c r="O3" s="45"/>
+    </row>
+    <row r="4" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="203" t="str">
         <f>RESUMEN!A13</f>
         <v>Importante para dueños o inquilinos de departamentos o coheras: Queremos recordarles una cuestión importante respecto a los pagos de expensas que ayuda a evitar errores en la imputación de los mismos. El sistema que utilizamos asigna centavos únicos a cada Unidad Funcional (UF), lo cual nos permite identificar automáticamente a qué unidad corresponde cada transferencia. Es decir, cada UF tiene un número específico de centavos que actúa como "identificador". Por ejemplo, si tu UF es la 45, el importe a abonar debería terminar en $...,45. Si tenés más de una unidad (por ejemplo, un departamento y una cochera), cada una tiene su propio código de centavos. En esos casos, te pedimos por favor que realices una transferencia por cada UF, respetando el importe con sus centavos correspondientes. Sabemos que a veces por comodidad se suele enviar todo junto en una sola transferencia, pero esto puede generar confusión o errores en la imputación automática. Realizar los pagos por separado nos permite asegurar que cada importe se asigne correctamente. Agradecemos muchísimo la colaboración para seguir manteniendo todo ordenado. Saludos cordiales.</v>
       </c>
-      <c r="B4" s="195"/>
-      <c r="C4" s="195"/>
-      <c r="D4" s="195"/>
-      <c r="E4" s="195"/>
-      <c r="F4" s="195"/>
-      <c r="G4" s="195"/>
-      <c r="H4" s="195"/>
-      <c r="I4" s="195"/>
-      <c r="J4" s="195"/>
-      <c r="K4" s="195"/>
-      <c r="L4" s="195"/>
-      <c r="M4" s="195"/>
-      <c r="N4" s="195"/>
-      <c r="O4" s="196"/>
-    </row>
-    <row r="5" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="197"/>
-      <c r="B5" s="198"/>
-      <c r="C5" s="198"/>
-      <c r="D5" s="198"/>
-      <c r="E5" s="198"/>
-      <c r="F5" s="198"/>
-      <c r="G5" s="198"/>
-      <c r="H5" s="198"/>
-      <c r="I5" s="198"/>
-      <c r="J5" s="198"/>
-      <c r="K5" s="198"/>
-      <c r="L5" s="198"/>
-      <c r="M5" s="198"/>
-      <c r="N5" s="198"/>
-      <c r="O5" s="199"/>
-    </row>
-    <row r="6" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="197"/>
-      <c r="B6" s="198"/>
-      <c r="C6" s="198"/>
-      <c r="D6" s="198"/>
-      <c r="E6" s="198"/>
-      <c r="F6" s="198"/>
-      <c r="G6" s="198"/>
-      <c r="H6" s="198"/>
-      <c r="I6" s="198"/>
-      <c r="J6" s="198"/>
-      <c r="K6" s="198"/>
-      <c r="L6" s="198"/>
-      <c r="M6" s="198"/>
-      <c r="N6" s="198"/>
-      <c r="O6" s="199"/>
-    </row>
-    <row r="7" spans="1:18" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="197"/>
-      <c r="B7" s="198"/>
-      <c r="C7" s="198"/>
-      <c r="D7" s="198"/>
-      <c r="E7" s="198"/>
-      <c r="F7" s="198"/>
-      <c r="G7" s="198"/>
-      <c r="H7" s="198"/>
-      <c r="I7" s="198"/>
-      <c r="J7" s="198"/>
-      <c r="K7" s="198"/>
-      <c r="L7" s="198"/>
-      <c r="M7" s="198"/>
-      <c r="N7" s="198"/>
-      <c r="O7" s="199"/>
-    </row>
-    <row r="8" spans="1:18" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="200"/>
-      <c r="B8" s="201"/>
-      <c r="C8" s="201"/>
-      <c r="D8" s="201"/>
-      <c r="E8" s="201"/>
-      <c r="F8" s="201"/>
-      <c r="G8" s="201"/>
-      <c r="H8" s="201"/>
-      <c r="I8" s="201"/>
-      <c r="J8" s="201"/>
-      <c r="K8" s="201"/>
-      <c r="L8" s="201"/>
-      <c r="M8" s="201"/>
-      <c r="N8" s="201"/>
-      <c r="O8" s="202"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="186" t="s">
+      <c r="B4" s="204"/>
+      <c r="C4" s="204"/>
+      <c r="D4" s="204"/>
+      <c r="E4" s="204"/>
+      <c r="F4" s="204"/>
+      <c r="G4" s="204"/>
+      <c r="H4" s="204"/>
+      <c r="I4" s="204"/>
+      <c r="J4" s="204"/>
+      <c r="K4" s="204"/>
+      <c r="L4" s="204"/>
+      <c r="M4" s="204"/>
+      <c r="N4" s="204"/>
+      <c r="O4" s="205"/>
+    </row>
+    <row r="5" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="206"/>
+      <c r="B5" s="207"/>
+      <c r="C5" s="207"/>
+      <c r="D5" s="207"/>
+      <c r="E5" s="207"/>
+      <c r="F5" s="207"/>
+      <c r="G5" s="207"/>
+      <c r="H5" s="207"/>
+      <c r="I5" s="207"/>
+      <c r="J5" s="207"/>
+      <c r="K5" s="207"/>
+      <c r="L5" s="207"/>
+      <c r="M5" s="207"/>
+      <c r="N5" s="207"/>
+      <c r="O5" s="208"/>
+    </row>
+    <row r="6" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="206"/>
+      <c r="B6" s="207"/>
+      <c r="C6" s="207"/>
+      <c r="D6" s="207"/>
+      <c r="E6" s="207"/>
+      <c r="F6" s="207"/>
+      <c r="G6" s="207"/>
+      <c r="H6" s="207"/>
+      <c r="I6" s="207"/>
+      <c r="J6" s="207"/>
+      <c r="K6" s="207"/>
+      <c r="L6" s="207"/>
+      <c r="M6" s="207"/>
+      <c r="N6" s="207"/>
+      <c r="O6" s="208"/>
+    </row>
+    <row r="7" spans="1:18" ht="64.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="206"/>
+      <c r="B7" s="207"/>
+      <c r="C7" s="207"/>
+      <c r="D7" s="207"/>
+      <c r="E7" s="207"/>
+      <c r="F7" s="207"/>
+      <c r="G7" s="207"/>
+      <c r="H7" s="207"/>
+      <c r="I7" s="207"/>
+      <c r="J7" s="207"/>
+      <c r="K7" s="207"/>
+      <c r="L7" s="207"/>
+      <c r="M7" s="207"/>
+      <c r="N7" s="207"/>
+      <c r="O7" s="208"/>
+    </row>
+    <row r="8" spans="1:18" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="209"/>
+      <c r="B8" s="210"/>
+      <c r="C8" s="210"/>
+      <c r="D8" s="210"/>
+      <c r="E8" s="210"/>
+      <c r="F8" s="210"/>
+      <c r="G8" s="210"/>
+      <c r="H8" s="210"/>
+      <c r="I8" s="210"/>
+      <c r="J8" s="210"/>
+      <c r="K8" s="210"/>
+      <c r="L8" s="210"/>
+      <c r="M8" s="210"/>
+      <c r="N8" s="210"/>
+      <c r="O8" s="211"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="195" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="188" t="s">
+      <c r="B9" s="189" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="188" t="s">
+      <c r="C9" s="189" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="120"/>
-      <c r="E9" s="188" t="s">
+      <c r="D9" s="119"/>
+      <c r="E9" s="189" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="186" t="s">
+      <c r="F9" s="195" t="s">
         <v>38</v>
       </c>
-      <c r="G9" s="188" t="s">
+      <c r="G9" s="218" t="s">
         <v>7</v>
       </c>
-      <c r="H9" s="188" t="s">
+      <c r="H9" s="189" t="s">
         <v>106</v>
       </c>
-      <c r="I9" s="190" t="s">
+      <c r="I9" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="186" t="s">
+      <c r="J9" s="195" t="s">
         <v>33</v>
       </c>
-      <c r="K9" s="186" t="s">
+      <c r="K9" s="195" t="s">
         <v>112</v>
       </c>
-      <c r="L9" s="186" t="s">
+      <c r="L9" s="195" t="s">
         <v>21</v>
       </c>
-      <c r="M9" s="192" t="s">
+      <c r="M9" s="201" t="s">
         <v>48</v>
       </c>
-      <c r="N9" s="48" t="s">
+      <c r="N9" s="47" t="s">
         <v>30</v>
       </c>
-      <c r="O9" s="205" t="s">
+      <c r="O9" s="213" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="203"/>
-      <c r="B10" s="204"/>
-      <c r="C10" s="189"/>
-      <c r="D10" s="121"/>
-      <c r="E10" s="189"/>
-      <c r="F10" s="187"/>
-      <c r="G10" s="189"/>
-      <c r="H10" s="204"/>
-      <c r="I10" s="191"/>
-      <c r="J10" s="187"/>
-      <c r="K10" s="187"/>
-      <c r="L10" s="187"/>
-      <c r="M10" s="193"/>
-      <c r="N10" s="47" t="str">
+    <row r="10" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="212"/>
+      <c r="B10" s="190"/>
+      <c r="C10" s="198"/>
+      <c r="D10" s="120"/>
+      <c r="E10" s="198"/>
+      <c r="F10" s="196"/>
+      <c r="G10" s="219"/>
+      <c r="H10" s="190"/>
+      <c r="I10" s="200"/>
+      <c r="J10" s="196"/>
+      <c r="K10" s="196"/>
+      <c r="L10" s="196"/>
+      <c r="M10" s="202"/>
+      <c r="N10" s="46" t="str">
         <f>RESUMEN!B8</f>
         <v>VTO 16/10</v>
       </c>
-      <c r="O10" s="206"/>
-    </row>
-    <row r="11" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="99" t="s">
+      <c r="O10" s="214"/>
+    </row>
+    <row r="11" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="98" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="99" t="s">
+      <c r="B11" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="99" t="s">
+      <c r="C11" s="98" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="99"/>
-      <c r="E11" s="118">
+      <c r="D11" s="98"/>
+      <c r="E11" s="117">
         <v>6.18</v>
       </c>
-      <c r="F11" s="101">
-        <v>286619.01</v>
-      </c>
-      <c r="G11" s="145">
+      <c r="F11" s="100">
+        <v>271124.01</v>
+      </c>
+      <c r="G11" s="144">
         <f>F11</f>
-        <v>286619.01</v>
-      </c>
-      <c r="H11" s="102" t="s">
+        <v>271124.01</v>
+      </c>
+      <c r="H11" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I11" s="103">
+      <c r="I11" s="102">
         <f t="shared" ref="I11:I35" si="0">F11-G11</f>
         <v>0</v>
       </c>
-      <c r="J11" s="103">
+      <c r="J11" s="102">
         <f>IF(I11&gt;0,I11*3%,0)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="103"/>
-      <c r="L11" s="104">
+      <c r="K11" s="102"/>
+      <c r="L11" s="103">
         <f>M$2*E11/100</f>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M11" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M11" s="104">
         <f>D$2*E11/100</f>
         <v>0</v>
       </c>
-      <c r="N11" s="106">
+      <c r="N11" s="105">
         <f t="shared" ref="N11:N35" si="1">ROUND(SUM(I11:M11),0) + P11</f>
-        <v>271124.01</v>
-      </c>
-      <c r="O11" s="107">
+        <v>270623.01</v>
+      </c>
+      <c r="O11" s="106">
         <f t="shared" ref="O11:O35" si="2">ROUND(N11*3%,0) + N11</f>
-        <v>279258.01</v>
+        <v>278742.01</v>
       </c>
       <c r="P11" s="33">
         <v>0.01</v>
       </c>
       <c r="Q11" s="33"/>
     </row>
-    <row r="12" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="99" t="s">
+    <row r="12" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="98" t="s">
         <v>51</v>
       </c>
-      <c r="B12" s="99" t="s">
+      <c r="B12" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="99" t="s">
+      <c r="C12" s="98" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="99" t="s">
+      <c r="D12" s="98" t="s">
         <v>101</v>
       </c>
-      <c r="E12" s="118">
+      <c r="E12" s="117">
         <v>4.33</v>
       </c>
-      <c r="F12" s="101">
-        <v>195652.02</v>
-      </c>
-      <c r="G12" s="109">
-        <v>201522.02</v>
-      </c>
-      <c r="H12" s="102" t="s">
+      <c r="F12" s="100">
+        <v>184092.02</v>
+      </c>
+      <c r="G12" s="108">
+        <v>189615.02</v>
+      </c>
+      <c r="H12" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I12" s="103">
+      <c r="I12" s="102">
         <f t="shared" si="0"/>
-        <v>-5870</v>
-      </c>
-      <c r="J12" s="103">
+        <v>-5523</v>
+      </c>
+      <c r="J12" s="102">
         <f t="shared" ref="J12:J35" si="3">IF(I12&gt;0,I12*3%,0)</f>
         <v>0</v>
       </c>
-      <c r="K12" s="103"/>
-      <c r="L12" s="104">
+      <c r="K12" s="102"/>
+      <c r="L12" s="103">
         <f t="shared" ref="L12:L35" si="4">M$2*E12/100</f>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M12" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M12" s="104">
         <f t="shared" ref="M12:M35" si="5">D$2*E12/100</f>
         <v>0</v>
       </c>
-      <c r="N12" s="106">
+      <c r="N12" s="105">
         <f t="shared" si="1"/>
-        <v>184092.02</v>
-      </c>
-      <c r="O12" s="107">
+        <v>184088.02</v>
+      </c>
+      <c r="O12" s="106">
         <f t="shared" si="2"/>
-        <v>189615.02</v>
+        <v>189611.02</v>
       </c>
       <c r="P12" s="33">
         <f>P11+0.01</f>
@@ -3370,54 +3378,54 @@
       </c>
       <c r="Q12" s="33"/>
     </row>
-    <row r="13" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="108" t="s">
+    <row r="13" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="107" t="s">
         <v>56</v>
       </c>
-      <c r="B13" s="108" t="s">
+      <c r="B13" s="107" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="108" t="s">
+      <c r="C13" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="D13" s="108"/>
-      <c r="E13" s="119">
+      <c r="D13" s="107"/>
+      <c r="E13" s="118">
         <v>6.18</v>
       </c>
-      <c r="F13" s="109">
-        <v>282092.03000000003</v>
-      </c>
-      <c r="G13" s="109">
-        <f>320000-G30</f>
-        <v>291278.8</v>
-      </c>
-      <c r="H13" s="102" t="s">
+      <c r="F13" s="108">
+        <v>261937.03</v>
+      </c>
+      <c r="G13" s="108">
+        <f>310000-G30</f>
+        <v>276087.8</v>
+      </c>
+      <c r="H13" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I13" s="103">
+      <c r="I13" s="102">
         <f t="shared" si="0"/>
-        <v>-9186.7699999999604</v>
-      </c>
-      <c r="J13" s="103">
+        <v>-14150.76999999999</v>
+      </c>
+      <c r="J13" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K13" s="103"/>
-      <c r="L13" s="104">
+      <c r="K13" s="102"/>
+      <c r="L13" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M13" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M13" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N13" s="106">
+      <c r="N13" s="105">
         <f t="shared" si="1"/>
-        <v>261937.03</v>
-      </c>
-      <c r="O13" s="107">
+        <v>256472.03</v>
+      </c>
+      <c r="O13" s="106">
         <f t="shared" si="2"/>
-        <v>269795.03000000003</v>
+        <v>264166.03000000003</v>
       </c>
       <c r="P13" s="33">
         <f t="shared" ref="P13:P35" si="6">P12+0.01</f>
@@ -3425,54 +3433,54 @@
       </c>
       <c r="Q13" s="32"/>
     </row>
-    <row r="14" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="99" t="s">
+    <row r="14" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="98" t="s">
         <v>56</v>
       </c>
-      <c r="B14" s="99" t="s">
+      <c r="B14" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="99" t="s">
+      <c r="C14" s="98" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="99"/>
-      <c r="E14" s="118">
+      <c r="D14" s="98"/>
+      <c r="E14" s="117">
         <v>4.33</v>
       </c>
-      <c r="F14" s="101">
-        <v>200818.04</v>
-      </c>
-      <c r="G14" s="109">
+      <c r="F14" s="100">
+        <v>189962.04</v>
+      </c>
+      <c r="G14" s="108">
         <f>F14</f>
-        <v>200818.04</v>
-      </c>
-      <c r="H14" s="102" t="s">
+        <v>189962.04</v>
+      </c>
+      <c r="H14" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I14" s="103">
+      <c r="I14" s="102">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J14" s="103">
+      <c r="J14" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K14" s="103"/>
-      <c r="L14" s="104">
+      <c r="K14" s="102"/>
+      <c r="L14" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M14" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M14" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N14" s="106">
+      <c r="N14" s="105">
         <f t="shared" si="1"/>
-        <v>189962.04</v>
-      </c>
-      <c r="O14" s="107">
+        <v>189611.04</v>
+      </c>
+      <c r="O14" s="106">
         <f t="shared" si="2"/>
-        <v>195661.04</v>
+        <v>195299.04</v>
       </c>
       <c r="P14" s="33">
         <f t="shared" si="6"/>
@@ -3480,56 +3488,56 @@
       </c>
       <c r="R14" s="33"/>
     </row>
-    <row r="15" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="99" t="s">
+    <row r="15" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="98" t="s">
         <v>59</v>
       </c>
-      <c r="B15" s="99" t="s">
+      <c r="B15" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="99" t="s">
+      <c r="C15" s="98" t="s">
         <v>60</v>
       </c>
-      <c r="D15" s="99" t="s">
+      <c r="D15" s="98" t="s">
         <v>100</v>
       </c>
-      <c r="E15" s="118">
+      <c r="E15" s="117">
         <v>6.18</v>
       </c>
-      <c r="F15" s="101">
-        <v>286619.05</v>
-      </c>
-      <c r="G15" s="109">
+      <c r="F15" s="100">
+        <v>271124.05</v>
+      </c>
+      <c r="G15" s="108">
         <f>F15</f>
-        <v>286619.05</v>
-      </c>
-      <c r="H15" s="102" t="s">
+        <v>271124.05</v>
+      </c>
+      <c r="H15" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I15" s="103">
+      <c r="I15" s="102">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J15" s="103">
+      <c r="J15" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K15" s="103"/>
-      <c r="L15" s="104">
+      <c r="K15" s="102"/>
+      <c r="L15" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M15" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M15" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N15" s="106">
+      <c r="N15" s="105">
         <f t="shared" si="1"/>
-        <v>271124.05</v>
-      </c>
-      <c r="O15" s="107">
+        <v>270623.05</v>
+      </c>
+      <c r="O15" s="106">
         <f t="shared" si="2"/>
-        <v>279258.05</v>
+        <v>278742.05</v>
       </c>
       <c r="P15" s="33">
         <f t="shared" si="6"/>
@@ -3537,1177 +3545,1178 @@
       </c>
       <c r="R15" s="33"/>
     </row>
-    <row r="16" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="99" t="s">
+    <row r="16" spans="1:18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="98" t="s">
         <v>59</v>
       </c>
-      <c r="B16" s="99" t="s">
+      <c r="B16" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="99" t="s">
+      <c r="C16" s="98" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="99"/>
-      <c r="E16" s="118">
+      <c r="D16" s="98"/>
+      <c r="E16" s="117">
         <v>4.33</v>
       </c>
-      <c r="F16" s="101">
-        <v>200818.06</v>
-      </c>
-      <c r="G16" s="109">
-        <f>F16</f>
-        <v>200818.06</v>
-      </c>
-      <c r="H16" s="102" t="s">
+      <c r="F16" s="100">
+        <v>189962.06</v>
+      </c>
+      <c r="G16" s="108">
+        <v>195655.06</v>
+      </c>
+      <c r="H16" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I16" s="103">
+      <c r="I16" s="102">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J16" s="103">
+        <v>-5693</v>
+      </c>
+      <c r="J16" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K16" s="103"/>
-      <c r="L16" s="104">
+      <c r="K16" s="102"/>
+      <c r="L16" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M16" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M16" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N16" s="106">
+      <c r="N16" s="105">
         <f t="shared" si="1"/>
-        <v>189962.06</v>
-      </c>
-      <c r="O16" s="107">
+        <v>183918.06</v>
+      </c>
+      <c r="O16" s="106">
         <f t="shared" si="2"/>
-        <v>195661.06</v>
+        <v>189436.06</v>
       </c>
       <c r="P16" s="33">
         <f t="shared" si="6"/>
         <v>6.0000000000000005E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="99" t="s">
+    <row r="17" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="98" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="99" t="s">
+      <c r="B17" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="99" t="s">
+      <c r="C17" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="99"/>
-      <c r="E17" s="118">
+      <c r="D17" s="98"/>
+      <c r="E17" s="117">
         <v>6.18</v>
       </c>
-      <c r="F17" s="101">
-        <v>261393.07</v>
-      </c>
-      <c r="G17" s="109">
-        <f>299000-G32</f>
-        <v>262072.78</v>
-      </c>
-      <c r="H17" s="102" t="s">
+      <c r="F17" s="100">
+        <v>270444.07</v>
+      </c>
+      <c r="G17" s="108">
+        <f>305000-G32</f>
+        <v>271087.78000000003</v>
+      </c>
+      <c r="H17" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I17" s="103">
+      <c r="I17" s="102">
         <f t="shared" si="0"/>
-        <v>-679.70999999999185</v>
-      </c>
-      <c r="J17" s="103">
+        <v>-643.71000000002095</v>
+      </c>
+      <c r="J17" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K17" s="103"/>
-      <c r="L17" s="104">
+      <c r="K17" s="102"/>
+      <c r="L17" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M17" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M17" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N17" s="106">
+      <c r="N17" s="105">
         <f t="shared" si="1"/>
-        <v>270444.07</v>
-      </c>
-      <c r="O17" s="107">
+        <v>269979.07</v>
+      </c>
+      <c r="O17" s="106">
         <f t="shared" si="2"/>
-        <v>278557.07</v>
+        <v>278078.07</v>
       </c>
       <c r="P17" s="33">
         <f t="shared" si="6"/>
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="99" t="s">
+    <row r="18" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="98" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="99" t="s">
+      <c r="B18" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="99" t="s">
+      <c r="C18" s="98" t="s">
         <v>64</v>
       </c>
-      <c r="D18" s="99"/>
-      <c r="E18" s="118">
+      <c r="D18" s="98"/>
+      <c r="E18" s="117">
         <v>4.33</v>
       </c>
-      <c r="F18" s="101">
-        <v>200818.08</v>
-      </c>
-      <c r="G18" s="109">
+      <c r="F18" s="100">
+        <v>189962.08</v>
+      </c>
+      <c r="G18" s="108">
         <f>F18</f>
-        <v>200818.08</v>
-      </c>
-      <c r="H18" s="102" t="s">
+        <v>189962.08</v>
+      </c>
+      <c r="H18" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I18" s="103">
+      <c r="I18" s="102">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J18" s="103">
+      <c r="J18" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K18" s="103"/>
-      <c r="L18" s="104">
+      <c r="K18" s="102"/>
+      <c r="L18" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M18" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M18" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N18" s="106">
+      <c r="N18" s="105">
         <f t="shared" si="1"/>
-        <v>189962.08</v>
-      </c>
-      <c r="O18" s="107">
+        <v>189611.08</v>
+      </c>
+      <c r="O18" s="106">
         <f t="shared" si="2"/>
-        <v>195661.08</v>
+        <v>195299.08</v>
       </c>
       <c r="P18" s="33">
         <f t="shared" si="6"/>
         <v>0.08</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="99" t="s">
+    <row r="19" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="99" t="s">
+      <c r="B19" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="99" t="s">
+      <c r="C19" s="98" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="99"/>
-      <c r="E19" s="118">
+      <c r="D19" s="98"/>
+      <c r="E19" s="117">
         <v>6.18</v>
       </c>
-      <c r="F19" s="101">
-        <v>189553.09</v>
-      </c>
-      <c r="G19" s="109">
-        <f>189553.09</f>
-        <v>189553.09</v>
-      </c>
-      <c r="H19" s="102" t="s">
+      <c r="F19" s="100">
+        <v>271124.09000000003</v>
+      </c>
+      <c r="G19" s="108">
+        <f>302032.34-G33</f>
+        <v>271124.11000000004</v>
+      </c>
+      <c r="H19" s="101" t="s">
         <v>107</v>
       </c>
-      <c r="I19" s="103">
+      <c r="I19" s="102">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J19" s="103">
+        <v>-2.0000000018626451E-2</v>
+      </c>
+      <c r="J19" s="102">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K19" s="103"/>
-      <c r="L19" s="104">
+      <c r="K19" s="102"/>
+      <c r="L19" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M19" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M19" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N19" s="106">
+      <c r="N19" s="105">
         <f>ROUND(SUM(I19:M19),0) + P19</f>
-        <v>271124.09000000003</v>
-      </c>
-      <c r="O19" s="107">
+        <v>270623.09000000003</v>
+      </c>
+      <c r="O19" s="106">
         <f t="shared" si="2"/>
-        <v>279258.09000000003</v>
+        <v>278742.09000000003</v>
       </c>
       <c r="P19" s="33">
         <f t="shared" si="6"/>
         <v>0.09</v>
       </c>
     </row>
-    <row r="20" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="99" t="s">
+    <row r="20" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="98" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="99" t="s">
+      <c r="B20" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C20" s="99" t="s">
+      <c r="C20" s="98" t="s">
         <v>67</v>
       </c>
-      <c r="D20" s="99"/>
-      <c r="E20" s="118">
+      <c r="D20" s="98"/>
+      <c r="E20" s="117">
         <v>4.33</v>
       </c>
-      <c r="F20" s="101">
-        <v>195654.1</v>
-      </c>
-      <c r="G20" s="109">
-        <v>195654</v>
-      </c>
-      <c r="H20" s="102" t="s">
+      <c r="F20" s="100">
+        <v>189962.1</v>
+      </c>
+      <c r="G20" s="108">
+        <f>F20</f>
+        <v>189962.1</v>
+      </c>
+      <c r="H20" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="I20" s="103">
+      <c r="I20" s="102">
         <f t="shared" si="0"/>
-        <v>0.10000000000582077</v>
-      </c>
-      <c r="J20" s="103">
+        <v>0</v>
+      </c>
+      <c r="J20" s="102">
         <f t="shared" si="3"/>
-        <v>3.000000000174623E-3</v>
-      </c>
-      <c r="K20" s="103"/>
-      <c r="L20" s="104">
+        <v>0</v>
+      </c>
+      <c r="K20" s="102"/>
+      <c r="L20" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M20" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M20" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N20" s="106">
+      <c r="N20" s="105">
         <f t="shared" si="1"/>
-        <v>189962.1</v>
-      </c>
-      <c r="O20" s="107">
+        <v>189611.1</v>
+      </c>
+      <c r="O20" s="106">
         <f t="shared" si="2"/>
-        <v>195661.1</v>
+        <v>195299.1</v>
       </c>
       <c r="P20" s="33">
         <f t="shared" si="6"/>
         <v>9.9999999999999992E-2</v>
       </c>
       <c r="Q20" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="99" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="99" t="s">
+      <c r="B21" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="99" t="s">
+      <c r="C21" s="98" t="s">
         <v>69</v>
       </c>
-      <c r="D21" s="99" t="s">
+      <c r="D21" s="98" t="s">
         <v>99</v>
       </c>
-      <c r="E21" s="118">
+      <c r="E21" s="117">
         <v>6.18</v>
       </c>
-      <c r="F21" s="101">
-        <v>286619.11</v>
-      </c>
-      <c r="G21" s="145">
+      <c r="F21" s="100">
+        <v>271124.11</v>
+      </c>
+      <c r="G21" s="144">
         <f>F21</f>
-        <v>286619.11</v>
-      </c>
-      <c r="H21" s="109" t="s">
+        <v>271124.11</v>
+      </c>
+      <c r="H21" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I21" s="154">
+      <c r="I21" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J21" s="154">
+      <c r="J21" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K21" s="103"/>
-      <c r="L21" s="104">
+      <c r="K21" s="102"/>
+      <c r="L21" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M21" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M21" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N21" s="106">
+      <c r="N21" s="105">
         <f t="shared" si="1"/>
-        <v>271124.11</v>
-      </c>
-      <c r="O21" s="107">
+        <v>270623.11</v>
+      </c>
+      <c r="O21" s="106">
         <f t="shared" si="2"/>
-        <v>279258.11</v>
+        <v>278742.11</v>
       </c>
       <c r="P21" s="33">
         <f t="shared" si="6"/>
         <v>0.10999999999999999</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="99" t="s">
+    <row r="22" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="99" t="s">
+      <c r="B22" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="99" t="s">
+      <c r="C22" s="98" t="s">
         <v>70</v>
       </c>
-      <c r="D22" s="99"/>
-      <c r="E22" s="118">
+      <c r="D22" s="98"/>
+      <c r="E22" s="117">
         <v>4.33</v>
       </c>
-      <c r="F22" s="101">
-        <v>195225.12</v>
-      </c>
-      <c r="G22" s="109">
-        <v>202000</v>
-      </c>
-      <c r="H22" s="109" t="s">
+      <c r="F22" s="100">
+        <v>183187.12</v>
+      </c>
+      <c r="G22" s="108">
+        <v>189000</v>
+      </c>
+      <c r="H22" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I22" s="154">
+      <c r="I22" s="153">
         <f t="shared" si="0"/>
-        <v>-6774.8800000000047</v>
-      </c>
-      <c r="J22" s="154">
+        <v>-5812.8800000000047</v>
+      </c>
+      <c r="J22" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K22" s="103"/>
-      <c r="L22" s="104">
+      <c r="K22" s="102"/>
+      <c r="L22" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M22" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M22" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N22" s="106">
+      <c r="N22" s="105">
         <f t="shared" si="1"/>
-        <v>183187.12</v>
-      </c>
-      <c r="O22" s="107">
+        <v>183799.12</v>
+      </c>
+      <c r="O22" s="106">
         <f t="shared" si="2"/>
-        <v>188683.12</v>
+        <v>189313.12</v>
       </c>
       <c r="P22" s="33">
         <f t="shared" si="6"/>
         <v>0.11999999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="99" t="s">
+    <row r="23" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="98" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="99" t="s">
+      <c r="B23" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="99" t="s">
+      <c r="C23" s="98" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="99" t="s">
+      <c r="D23" s="98" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="118">
+      <c r="E23" s="117">
         <v>6.18</v>
       </c>
-      <c r="F23" s="101">
-        <v>295218.13</v>
-      </c>
-      <c r="G23" s="109">
+      <c r="F23" s="100">
+        <v>279258.13</v>
+      </c>
+      <c r="G23" s="108">
         <f>F23</f>
-        <v>295218.13</v>
-      </c>
-      <c r="H23" s="109" t="s">
+        <v>279258.13</v>
+      </c>
+      <c r="H23" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I23" s="154">
+      <c r="I23" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J23" s="154">
+      <c r="J23" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K23" s="103"/>
-      <c r="L23" s="104">
+      <c r="K23" s="102"/>
+      <c r="L23" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M23" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M23" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N23" s="106">
+      <c r="N23" s="105">
         <f t="shared" si="1"/>
-        <v>271124.13</v>
-      </c>
-      <c r="O23" s="107">
+        <v>270623.13</v>
+      </c>
+      <c r="O23" s="106">
         <f t="shared" si="2"/>
-        <v>279258.13</v>
+        <v>278742.13</v>
       </c>
       <c r="P23" s="33">
         <f t="shared" si="6"/>
         <v>0.12999999999999998</v>
       </c>
     </row>
-    <row r="24" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="99" t="s">
+    <row r="24" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="98" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="99" t="s">
+      <c r="B24" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="99" t="s">
+      <c r="C24" s="98" t="s">
         <v>73</v>
       </c>
-      <c r="D24" s="99"/>
-      <c r="E24" s="118">
+      <c r="D24" s="98"/>
+      <c r="E24" s="117">
         <v>4.33</v>
       </c>
-      <c r="F24" s="101">
-        <v>200818.14</v>
-      </c>
-      <c r="G24" s="109">
-        <v>206843.14</v>
-      </c>
-      <c r="H24" s="109" t="s">
+      <c r="F24" s="100">
+        <v>183937.14</v>
+      </c>
+      <c r="G24" s="144">
+        <f>F24</f>
+        <v>183937.14</v>
+      </c>
+      <c r="H24" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I24" s="154">
+      <c r="I24" s="153">
         <f t="shared" si="0"/>
-        <v>-6025</v>
-      </c>
-      <c r="J24" s="154">
+        <v>0</v>
+      </c>
+      <c r="J24" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K24" s="103"/>
-      <c r="L24" s="104">
+      <c r="K24" s="102"/>
+      <c r="L24" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M24" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M24" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N24" s="106">
+      <c r="N24" s="105">
         <f t="shared" si="1"/>
-        <v>183937.14</v>
-      </c>
-      <c r="O24" s="107">
+        <v>189611.14</v>
+      </c>
+      <c r="O24" s="106">
         <f t="shared" si="2"/>
-        <v>189455.14</v>
+        <v>195299.14</v>
       </c>
       <c r="P24" s="33">
         <f t="shared" si="6"/>
         <v>0.13999999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="108" t="s">
+    <row r="25" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="107" t="s">
         <v>74</v>
       </c>
-      <c r="B25" s="108" t="s">
+      <c r="B25" s="107" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="108" t="s">
+      <c r="C25" s="107" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="108"/>
-      <c r="E25" s="119">
+      <c r="D25" s="107"/>
+      <c r="E25" s="118">
         <v>6.18</v>
       </c>
-      <c r="F25" s="109">
-        <v>286619.15000000002</v>
-      </c>
-      <c r="G25" s="109">
-        <f>466282.97-G26-G35</f>
-        <v>229613.55999999994</v>
-      </c>
-      <c r="H25" s="109" t="s">
+      <c r="F25" s="108">
+        <v>329840.15000000002</v>
+      </c>
+      <c r="G25" s="108">
+        <f>553714.86-G26-G35</f>
+        <v>329840.44999999995</v>
+      </c>
+      <c r="H25" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I25" s="154">
+      <c r="I25" s="153">
         <f t="shared" si="0"/>
-        <v>57005.590000000084</v>
-      </c>
-      <c r="J25" s="154">
+        <v>-0.29999999993015081</v>
+      </c>
+      <c r="J25" s="153">
         <f t="shared" si="3"/>
-        <v>1710.1677000000025</v>
-      </c>
-      <c r="K25" s="103"/>
-      <c r="L25" s="104">
+        <v>0</v>
+      </c>
+      <c r="K25" s="102"/>
+      <c r="L25" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M25" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M25" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N25" s="106">
+      <c r="N25" s="105">
         <f t="shared" si="1"/>
-        <v>329840.15000000002</v>
-      </c>
-      <c r="O25" s="107">
+        <v>270623.15000000002</v>
+      </c>
+      <c r="O25" s="106">
         <f t="shared" si="2"/>
-        <v>339735.15</v>
+        <v>278742.15000000002</v>
       </c>
       <c r="P25" s="33">
         <f t="shared" si="6"/>
         <v>0.15</v>
       </c>
     </row>
-    <row r="26" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="99" t="s">
+    <row r="26" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="98" t="s">
         <v>74</v>
       </c>
-      <c r="B26" s="99" t="s">
+      <c r="B26" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="99" t="s">
+      <c r="C26" s="98" t="s">
         <v>75</v>
       </c>
-      <c r="D26" s="99"/>
-      <c r="E26" s="118">
+      <c r="D26" s="98"/>
+      <c r="E26" s="117">
         <v>4.33</v>
       </c>
-      <c r="F26" s="101">
-        <v>200818.16</v>
-      </c>
-      <c r="G26" s="109">
+      <c r="F26" s="100">
+        <v>189962.16</v>
+      </c>
+      <c r="G26" s="108">
         <f t="shared" ref="G26:G31" si="7">F26</f>
-        <v>200818.16</v>
-      </c>
-      <c r="H26" s="109" t="s">
+        <v>189962.16</v>
+      </c>
+      <c r="H26" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I26" s="154">
+      <c r="I26" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J26" s="154">
+      <c r="J26" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K26" s="103"/>
-      <c r="L26" s="104">
+      <c r="K26" s="102"/>
+      <c r="L26" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M26" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M26" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N26" s="106">
+      <c r="N26" s="105">
         <f t="shared" si="1"/>
-        <v>189962.16</v>
-      </c>
-      <c r="O26" s="107">
+        <v>189611.16</v>
+      </c>
+      <c r="O26" s="106">
         <f t="shared" si="2"/>
-        <v>195661.16</v>
+        <v>195299.16</v>
       </c>
       <c r="P26" s="33">
         <f t="shared" si="6"/>
         <v>0.16</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="99" t="s">
+    <row r="27" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="98" t="s">
         <v>76</v>
       </c>
-      <c r="B27" s="99" t="s">
+      <c r="B27" s="98" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="99" t="s">
+      <c r="C27" s="98" t="s">
         <v>77</v>
       </c>
-      <c r="D27" s="99" t="s">
+      <c r="D27" s="98" t="s">
         <v>102</v>
       </c>
-      <c r="E27" s="118">
+      <c r="E27" s="117">
         <v>6.18</v>
       </c>
-      <c r="F27" s="109">
-        <v>286619.17</v>
-      </c>
-      <c r="G27" s="109">
-        <f t="shared" si="7"/>
-        <v>286619.17</v>
-      </c>
-      <c r="H27" s="109" t="s">
+      <c r="F27" s="108">
+        <v>271124.17</v>
+      </c>
+      <c r="G27" s="108">
+        <f>F27</f>
+        <v>271124.17</v>
+      </c>
+      <c r="H27" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I27" s="154">
+      <c r="I27" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J27" s="154">
+      <c r="J27" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K27" s="103"/>
-      <c r="L27" s="104">
+      <c r="K27" s="102"/>
+      <c r="L27" s="103">
         <f t="shared" si="4"/>
-        <v>271124.07347399998</v>
-      </c>
-      <c r="M27" s="105">
+        <v>270623.17829400004</v>
+      </c>
+      <c r="M27" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N27" s="106">
+      <c r="N27" s="105">
         <f t="shared" si="1"/>
-        <v>271124.17</v>
-      </c>
-      <c r="O27" s="107">
+        <v>270623.17</v>
+      </c>
+      <c r="O27" s="106">
         <f t="shared" si="2"/>
-        <v>279258.17</v>
+        <v>278742.17</v>
       </c>
       <c r="P27" s="33">
         <f t="shared" si="6"/>
         <v>0.17</v>
       </c>
     </row>
-    <row r="28" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="99" t="s">
+    <row r="28" spans="1:17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="98" t="s">
         <v>76</v>
       </c>
-      <c r="B28" s="99" t="s">
+      <c r="B28" s="98" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="99" t="s">
+      <c r="C28" s="98" t="s">
         <v>78</v>
       </c>
-      <c r="D28" s="99"/>
-      <c r="E28" s="118">
+      <c r="D28" s="98"/>
+      <c r="E28" s="117">
         <v>4.33</v>
       </c>
-      <c r="F28" s="101">
-        <v>200818.18</v>
-      </c>
-      <c r="G28" s="145">
+      <c r="F28" s="100">
+        <v>189962.18</v>
+      </c>
+      <c r="G28" s="108">
         <f t="shared" si="7"/>
-        <v>200818.18</v>
-      </c>
-      <c r="H28" s="109" t="s">
+        <v>189962.18</v>
+      </c>
+      <c r="H28" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I28" s="154">
+      <c r="I28" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J28" s="154">
+      <c r="J28" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K28" s="103"/>
-      <c r="L28" s="104">
+      <c r="K28" s="102"/>
+      <c r="L28" s="103">
         <f t="shared" si="4"/>
-        <v>189962.33626899999</v>
-      </c>
-      <c r="M28" s="105">
+        <v>189611.38543900006</v>
+      </c>
+      <c r="M28" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N28" s="106">
+      <c r="N28" s="105">
         <f t="shared" si="1"/>
-        <v>189962.18</v>
-      </c>
-      <c r="O28" s="107">
+        <v>189611.18</v>
+      </c>
+      <c r="O28" s="106">
         <f t="shared" si="2"/>
-        <v>195661.18</v>
+        <v>195299.18</v>
       </c>
       <c r="P28" s="33">
         <f t="shared" si="6"/>
         <v>0.18000000000000002</v>
       </c>
     </row>
-    <row r="29" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="212" t="s">
+    <row r="29" spans="1:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="191" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="213"/>
-      <c r="C29" s="99" t="s">
+      <c r="B29" s="192"/>
+      <c r="C29" s="98" t="s">
         <v>77</v>
       </c>
-      <c r="D29" s="99"/>
-      <c r="E29" s="118">
+      <c r="D29" s="98"/>
+      <c r="E29" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F29" s="101">
-        <v>35851.19</v>
-      </c>
-      <c r="G29" s="109">
-        <f t="shared" si="7"/>
-        <v>35851.19</v>
-      </c>
-      <c r="H29" s="109" t="s">
+      <c r="F29" s="100">
+        <v>33912.19</v>
+      </c>
+      <c r="G29" s="108">
+        <f>F29</f>
+        <v>33912.19</v>
+      </c>
+      <c r="H29" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I29" s="154">
+      <c r="I29" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J29" s="154">
+      <c r="J29" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K29" s="103"/>
-      <c r="L29" s="104">
+      <c r="K29" s="102"/>
+      <c r="L29" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M29" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M29" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N29" s="106">
+      <c r="N29" s="105">
         <f t="shared" si="1"/>
-        <v>33912.19</v>
-      </c>
-      <c r="O29" s="107">
+        <v>33850.19</v>
+      </c>
+      <c r="O29" s="106">
         <f t="shared" si="2"/>
-        <v>34929.19</v>
+        <v>34866.19</v>
       </c>
       <c r="P29" s="33">
         <f t="shared" si="6"/>
         <v>0.19000000000000003</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="212" t="s">
+    <row r="30" spans="1:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="191" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="213"/>
-      <c r="C30" s="108" t="s">
+      <c r="B30" s="192"/>
+      <c r="C30" s="107" t="s">
         <v>57</v>
       </c>
-      <c r="D30" s="99"/>
-      <c r="E30" s="118">
+      <c r="D30" s="98"/>
+      <c r="E30" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F30" s="110">
-        <v>28721.200000000001</v>
-      </c>
-      <c r="G30" s="145">
+      <c r="F30" s="109">
+        <v>33912.199999999997</v>
+      </c>
+      <c r="G30" s="144">
         <f t="shared" si="7"/>
-        <v>28721.200000000001</v>
-      </c>
-      <c r="H30" s="109" t="s">
+        <v>33912.199999999997</v>
+      </c>
+      <c r="H30" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I30" s="154">
+      <c r="I30" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J30" s="154">
+      <c r="J30" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K30" s="103"/>
-      <c r="L30" s="104">
+      <c r="K30" s="102"/>
+      <c r="L30" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M30" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M30" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N30" s="106">
+      <c r="N30" s="105">
         <f t="shared" si="1"/>
-        <v>33912.199999999997</v>
-      </c>
-      <c r="O30" s="107">
+        <v>33850.199999999997</v>
+      </c>
+      <c r="O30" s="106">
         <f t="shared" si="2"/>
-        <v>34929.199999999997</v>
+        <v>34866.199999999997</v>
       </c>
       <c r="P30" s="33">
         <f t="shared" si="6"/>
         <v>0.20000000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="212" t="s">
+    <row r="31" spans="1:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="191" t="s">
         <v>82</v>
       </c>
-      <c r="B31" s="213"/>
-      <c r="C31" s="111" t="s">
+      <c r="B31" s="192"/>
+      <c r="C31" s="110" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="99" t="s">
+      <c r="D31" s="98" t="s">
         <v>104</v>
       </c>
-      <c r="E31" s="118">
+      <c r="E31" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F31" s="110">
-        <v>36927.21</v>
-      </c>
-      <c r="G31" s="145">
+      <c r="F31" s="109">
+        <v>34929.21</v>
+      </c>
+      <c r="G31" s="144">
         <f t="shared" si="7"/>
-        <v>36927.21</v>
-      </c>
-      <c r="H31" s="109" t="s">
+        <v>34929.21</v>
+      </c>
+      <c r="H31" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I31" s="154">
+      <c r="I31" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J31" s="154">
+      <c r="J31" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K31" s="103"/>
-      <c r="L31" s="104">
+      <c r="K31" s="102"/>
+      <c r="L31" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M31" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M31" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N31" s="106">
+      <c r="N31" s="105">
         <f t="shared" si="1"/>
-        <v>33912.21</v>
-      </c>
-      <c r="O31" s="107">
+        <v>33850.21</v>
+      </c>
+      <c r="O31" s="106">
         <f t="shared" si="2"/>
-        <v>34929.21</v>
+        <v>34866.21</v>
       </c>
       <c r="P31" s="33">
         <f t="shared" si="6"/>
         <v>0.21000000000000005</v>
       </c>
     </row>
-    <row r="32" spans="1:17" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="212" t="s">
+    <row r="32" spans="1:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="191" t="s">
         <v>83</v>
       </c>
-      <c r="B32" s="213"/>
-      <c r="C32" s="99" t="s">
+      <c r="B32" s="192"/>
+      <c r="C32" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="99"/>
-      <c r="E32" s="118">
+      <c r="D32" s="98"/>
+      <c r="E32" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F32" s="110">
-        <v>36927.22</v>
-      </c>
-      <c r="G32" s="145">
+      <c r="F32" s="109">
+        <v>33912.22</v>
+      </c>
+      <c r="G32" s="144">
         <f t="shared" ref="G32" si="8">F32</f>
-        <v>36927.22</v>
-      </c>
-      <c r="H32" s="109" t="s">
+        <v>33912.22</v>
+      </c>
+      <c r="H32" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I32" s="154">
+      <c r="I32" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J32" s="154">
+      <c r="J32" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K32" s="103"/>
-      <c r="L32" s="104">
+      <c r="K32" s="102"/>
+      <c r="L32" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M32" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M32" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N32" s="106">
+      <c r="N32" s="105">
         <f t="shared" si="1"/>
-        <v>33912.22</v>
-      </c>
-      <c r="O32" s="107">
+        <v>33850.22</v>
+      </c>
+      <c r="O32" s="106">
         <f t="shared" si="2"/>
-        <v>34929.22</v>
+        <v>34866.22</v>
       </c>
       <c r="P32" s="33">
         <f t="shared" si="6"/>
         <v>0.22000000000000006</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="212" t="s">
+    <row r="33" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="191" t="s">
         <v>84</v>
       </c>
-      <c r="B33" s="213"/>
-      <c r="C33" s="112" t="s">
+      <c r="B33" s="192"/>
+      <c r="C33" s="111" t="s">
         <v>66</v>
       </c>
-      <c r="D33" s="112"/>
-      <c r="E33" s="118">
+      <c r="D33" s="111"/>
+      <c r="E33" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F33" s="110">
-        <v>33923.230000000003</v>
-      </c>
-      <c r="G33" s="145">
-        <f>G32</f>
-        <v>36927.22</v>
-      </c>
-      <c r="H33" s="109" t="s">
+      <c r="F33" s="109">
+        <v>30908.23</v>
+      </c>
+      <c r="G33" s="144">
+        <f>F33</f>
+        <v>30908.23</v>
+      </c>
+      <c r="H33" s="108" t="s">
         <v>107</v>
       </c>
-      <c r="I33" s="154">
+      <c r="I33" s="153">
         <f t="shared" si="0"/>
-        <v>-3003.989999999998</v>
-      </c>
-      <c r="J33" s="154">
+        <v>0</v>
+      </c>
+      <c r="J33" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K33" s="103"/>
-      <c r="L33" s="104">
+      <c r="K33" s="102"/>
+      <c r="L33" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M33" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M33" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N33" s="106">
+      <c r="N33" s="105">
         <f t="shared" si="1"/>
-        <v>30908.23</v>
-      </c>
-      <c r="O33" s="107">
+        <v>33850.230000000003</v>
+      </c>
+      <c r="O33" s="106">
         <f t="shared" si="2"/>
-        <v>31835.23</v>
+        <v>34866.230000000003</v>
       </c>
       <c r="P33" s="33">
         <f t="shared" si="6"/>
         <v>0.23000000000000007</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="212" t="s">
+    <row r="34" spans="1:16" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="191" t="s">
         <v>85</v>
       </c>
-      <c r="B34" s="213"/>
-      <c r="C34" s="112" t="s">
+      <c r="B34" s="192"/>
+      <c r="C34" s="111" t="s">
         <v>69</v>
       </c>
-      <c r="D34" s="112" t="s">
+      <c r="D34" s="111" t="s">
         <v>114</v>
       </c>
-      <c r="E34" s="118">
+      <c r="E34" s="117">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F34" s="110">
-        <v>36829.24</v>
-      </c>
-      <c r="G34" s="145">
-        <v>45757</v>
-      </c>
-      <c r="H34" s="109" t="s">
+      <c r="F34" s="109">
+        <v>24985.24</v>
+      </c>
+      <c r="G34" s="144">
+        <v>0</v>
+      </c>
+      <c r="H34" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I34" s="154">
+      <c r="I34" s="153">
         <f t="shared" si="0"/>
-        <v>-8927.760000000002</v>
-      </c>
-      <c r="J34" s="154">
+        <v>24985.24</v>
+      </c>
+      <c r="J34" s="153">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K34" s="103"/>
-      <c r="L34" s="104">
+        <v>749.55719999999997</v>
+      </c>
+      <c r="K34" s="102"/>
+      <c r="L34" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M34" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M34" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N34" s="106">
+      <c r="N34" s="105">
         <f t="shared" si="1"/>
-        <v>24985.24</v>
-      </c>
-      <c r="O34" s="107">
+        <v>59585.24</v>
+      </c>
+      <c r="O34" s="106">
         <f t="shared" si="2"/>
-        <v>25735.24</v>
+        <v>61373.24</v>
       </c>
       <c r="P34" s="33">
         <f t="shared" si="6"/>
         <v>0.24000000000000007</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="212" t="s">
+    <row r="35" spans="1:16" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="191" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="213"/>
-      <c r="C35" s="112" t="s">
+      <c r="B35" s="192"/>
+      <c r="C35" s="111" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="112"/>
-      <c r="E35" s="100">
+      <c r="D35" s="111"/>
+      <c r="E35" s="99">
         <v>0.77300000000000002</v>
       </c>
-      <c r="F35" s="110">
-        <v>35851.25</v>
-      </c>
-      <c r="G35" s="109">
+      <c r="F35" s="109">
+        <v>33912.25</v>
+      </c>
+      <c r="G35" s="215">
         <f>F35</f>
-        <v>35851.25</v>
-      </c>
-      <c r="H35" s="109" t="s">
+        <v>33912.25</v>
+      </c>
+      <c r="H35" s="108" t="s">
         <v>54</v>
       </c>
-      <c r="I35" s="154">
+      <c r="I35" s="153">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J35" s="154">
+      <c r="J35" s="153">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K35" s="103"/>
-      <c r="L35" s="104">
+      <c r="K35" s="102"/>
+      <c r="L35" s="103">
         <f t="shared" si="4"/>
-        <v>33912.4447889</v>
-      </c>
-      <c r="M35" s="105">
+        <v>33849.792365900008</v>
+      </c>
+      <c r="M35" s="104">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N35" s="106">
+      <c r="N35" s="105">
         <f t="shared" si="1"/>
-        <v>33912.25</v>
-      </c>
-      <c r="O35" s="107">
+        <v>33850.25</v>
+      </c>
+      <c r="O35" s="106">
         <f t="shared" si="2"/>
-        <v>34929.25</v>
+        <v>34866.25</v>
       </c>
       <c r="P35" s="33">
         <f t="shared" si="6"/>
         <v>0.25000000000000006</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="214" t="s">
+    <row r="36" spans="1:16" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="193" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="214"/>
-      <c r="C36" s="215"/>
-      <c r="D36" s="122"/>
-      <c r="E36" s="113">
+      <c r="B36" s="193"/>
+      <c r="C36" s="194"/>
+      <c r="D36" s="121"/>
+      <c r="E36" s="112">
         <f t="shared" ref="E36:M36" si="9">SUM(E11:E35)</f>
         <v>100.00099999999993</v>
       </c>
-      <c r="F36" s="114">
+      <c r="F36" s="113">
         <f t="shared" si="9"/>
-        <v>4497822.2500000009</v>
-      </c>
-      <c r="G36" s="115">
+        <v>4414560.2500000009</v>
+      </c>
+      <c r="G36" s="114">
         <f t="shared" si="9"/>
-        <v>4481284.67</v>
-      </c>
-      <c r="H36" s="115"/>
-      <c r="I36" s="115">
+        <v>4421398.6900000004</v>
+      </c>
+      <c r="H36" s="114"/>
+      <c r="I36" s="114">
         <f t="shared" si="9"/>
-        <v>16537.580000000133</v>
-      </c>
-      <c r="J36" s="116">
+        <v>-6838.4399999999623</v>
+      </c>
+      <c r="J36" s="115">
         <f t="shared" si="9"/>
-        <v>1710.1707000000026</v>
-      </c>
-      <c r="K36" s="116"/>
-      <c r="L36" s="116">
+        <v>749.55719999999997</v>
+      </c>
+      <c r="K36" s="115"/>
+      <c r="L36" s="115">
         <f t="shared" si="9"/>
-        <v>4387164.8012093008</v>
-      </c>
-      <c r="M36" s="115">
+        <v>4379059.6201583035</v>
+      </c>
+      <c r="M36" s="114">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="N36" s="117">
+      <c r="N36" s="116">
         <f>SUM(N11:N28)</f>
-        <v>4179954.7100000004</v>
-      </c>
-      <c r="O36" s="117">
+        <v>4110284.7100000004</v>
+      </c>
+      <c r="O36" s="116">
         <f>SUM(O11:O35)</f>
-        <v>4537572.2500000009</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="39"/>
-      <c r="D37" s="39"/>
+        <v>4504164.2500000009</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
       <c r="F37" t="s">
         <v>109</v>
       </c>
-      <c r="G37" s="129">
+      <c r="G37" s="128">
         <f>SUMIF(H11:H35,"B",G11:G35)</f>
-        <v>4254804.3600000013</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A38" s="207"/>
-      <c r="B38" s="207"/>
-      <c r="E38" s="208"/>
-      <c r="F38" s="209" t="s">
+        <v>4119366.350000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A38" s="184"/>
+      <c r="B38" s="184"/>
+      <c r="E38" s="185"/>
+      <c r="F38" s="186" t="s">
         <v>110</v>
       </c>
-      <c r="G38" s="129">
+      <c r="G38" s="128">
         <f>SUMIF(H11:H35,"E",G11:G35)</f>
-        <v>226480.31</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A39" s="207"/>
-      <c r="B39" s="207"/>
-      <c r="E39" s="208"/>
-      <c r="F39" s="209"/>
-      <c r="G39" s="130">
+        <v>302032.34000000003</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A39" s="184"/>
+      <c r="B39" s="184"/>
+      <c r="E39" s="185"/>
+      <c r="F39" s="186"/>
+      <c r="G39" s="129">
         <f>SUM(G37:G38)</f>
-        <v>4481284.6700000009</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+        <v>4421398.6900000013</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F50">
         <f>SUM(E48:E49)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F54">
         <f>SUM(E52:E53)</f>
         <v>0</v>
@@ -4715,6 +4724,19 @@
     </row>
   </sheetData>
   <mergeCells count="29">
+    <mergeCell ref="E1:N1"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="A4:O8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="O9:O10"/>
     <mergeCell ref="A38:B39"/>
     <mergeCell ref="E38:E39"/>
     <mergeCell ref="F38:F39"/>
@@ -4731,19 +4753,6 @@
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="K9:K10"/>
-    <mergeCell ref="E1:N1"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="A4:O8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="O9:O10"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4754,7 +4763,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D7123E2-E76E-40B2-9631-974509386176}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>